<commit_message>
Refresh Kip's persistent continuity tracker through Episode 2
</commit_message>
<xml_diff>
--- a/projects/kip-quillman/continuity.xlsx
+++ b/projects/kip-quillman/continuity.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planned state" sheetId="1" r:id="R014d8179a0f3475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mana events" sheetId="2" r:id="Rdf07123fc7f543ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="XP events" sheetId="3" r:id="Rd48f8fff7b9b48e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story carryover" sheetId="4" r:id="Rdee0794d30d94512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed state" sheetId="5" r:id="Rbfc6b032082f43ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="6" r:id="Rfbf6047475504fac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planned state" sheetId="1" r:id="Ra0233dd2cb584fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mana events" sheetId="2" r:id="R7f536282d4474739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="XP events" sheetId="3" r:id="R3c0a0487986648ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story carryover" sheetId="4" r:id="R2ab9c7d053404d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed state" sheetId="5" r:id="R9a7194b063e54374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="6" r:id="R013d1f9918664e2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +66,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,6 +96,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8F6FA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -164,7 +179,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -440,11 +455,39 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="8">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -496,6 +539,17 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C2430"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE9EC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -623,7 +677,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="StoryCarryover" displayName="StoryCarryover" ref="A7:F1579" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="StoryCarryover" displayName="StoryCarryover" ref="A7:F1743" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Record ID"/>
     <x:tableColumn id="2" name="Ch"/>
@@ -960,7 +1014,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>Author plan. Latest confirmed Episode 1; next Episode 2. See Confirmed state.</x:v>
+        <x:v>Author plan. Latest confirmed Episode 2; next Episode 3. See Confirmed state.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -5875,7 +5929,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15c3f4f2d924786"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R157fad8573d04547"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16298,7 +16352,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R589928004a684c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eb76fb7e9034c08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20751,7 +20805,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6772d95ed54b4170"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c5ef54f2cd44bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52133,13 +52187,3293 @@
         <x:v>Confirmed from final text</x:v>
       </x:c>
     </x:row>
+    <x:row r="1580" ht="30" customHeight="1">
+      <x:c r="A1580" s="95" t="str">
+        <x:v>ACT-002-title</x:v>
+      </x:c>
+      <x:c r="B1580" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1580" s="95" t="str">
+        <x:v>Actual title</x:v>
+      </x:c>
+      <x:c r="D1580" s="96" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="E1580" s="96" t="str">
+        <x:v>Twenty Mana Left</x:v>
+      </x:c>
+      <x:c r="F1580" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1581" ht="30" customHeight="1">
+      <x:c r="A1581" s="99" t="str">
+        <x:v>ACT-002-source_file</x:v>
+      </x:c>
+      <x:c r="B1581" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1581" s="99" t="str">
+        <x:v>Actual source_file</x:v>
+      </x:c>
+      <x:c r="D1581" s="100" t="str">
+        <x:v>source_file</x:v>
+      </x:c>
+      <x:c r="E1581" s="100" t="str">
+        <x:v>chapters/chapter-01/episode-002.txt</x:v>
+      </x:c>
+      <x:c r="F1581" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1582" ht="30" customHeight="1">
+      <x:c r="A1582" s="95" t="str">
+        <x:v>ACT-002-source_sha256</x:v>
+      </x:c>
+      <x:c r="B1582" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1582" s="95" t="str">
+        <x:v>Actual source_sha256</x:v>
+      </x:c>
+      <x:c r="D1582" s="96" t="str">
+        <x:v>source_sha256</x:v>
+      </x:c>
+      <x:c r="E1582" s="96" t="str">
+        <x:v>be408ba46776ec799bef78564c6ba621f3193fc6bf9c10d2a66dd2e29f18202b</x:v>
+      </x:c>
+      <x:c r="F1582" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1583" ht="32" customHeight="1">
+      <x:c r="A1583" s="99" t="str">
+        <x:v>ACT-002-time</x:v>
+      </x:c>
+      <x:c r="B1583" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1583" s="99" t="str">
+        <x:v>Actual time</x:v>
+      </x:c>
+      <x:c r="D1583" s="100" t="str">
+        <x:v>time</x:v>
+      </x:c>
+      <x:c r="E1583" s="100" t="str">
+        <x:v>Same opening retreat, then protected wound treatment for twenty seconds and several minutes of active patient repositioning/room checks. No completed sitting/lying quiet recovery minute established.</x:v>
+      </x:c>
+      <x:c r="F1583" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1584" ht="48" customHeight="1">
+      <x:c r="A1584" s="95" t="str">
+        <x:v>ACT-002-location</x:v>
+      </x:c>
+      <x:c r="B1584" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1584" s="95" t="str">
+        <x:v>Actual location</x:v>
+      </x:c>
+      <x:c r="D1584" s="96" t="str">
+        <x:v>location</x:v>
+      </x:c>
+      <x:c r="E1584" s="96" t="str">
+        <x:v>All five inside the old service chamber, approximately twelve by ten metres. Entry door closed and barred; second service passage obstructed by fallen stone. Intact squat anchor near the middle of the floor, not yet inspected or claimed.</x:v>
+      </x:c>
+      <x:c r="F1584" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1585" ht="30" customHeight="1">
+      <x:c r="A1585" s="99" t="str">
+        <x:v>ACT-002-roster.001</x:v>
+      </x:c>
+      <x:c r="B1585" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1585" s="99" t="str">
+        <x:v>Actual roster</x:v>
+      </x:c>
+      <x:c r="D1585" s="100" t="str">
+        <x:v>roster.001</x:v>
+      </x:c>
+      <x:c r="E1585" s="100" t="str">
+        <x:v>Kip Quillman</x:v>
+      </x:c>
+      <x:c r="F1585" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1586" ht="30" customHeight="1">
+      <x:c r="A1586" s="95" t="str">
+        <x:v>ACT-002-roster.002</x:v>
+      </x:c>
+      <x:c r="B1586" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1586" s="95" t="str">
+        <x:v>Actual roster</x:v>
+      </x:c>
+      <x:c r="D1586" s="96" t="str">
+        <x:v>roster.002</x:v>
+      </x:c>
+      <x:c r="E1586" s="96" t="str">
+        <x:v>Tessa Ward</x:v>
+      </x:c>
+      <x:c r="F1586" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1587" ht="30" customHeight="1">
+      <x:c r="A1587" s="99" t="str">
+        <x:v>ACT-002-roster.003</x:v>
+      </x:c>
+      <x:c r="B1587" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1587" s="99" t="str">
+        <x:v>Actual roster</x:v>
+      </x:c>
+      <x:c r="D1587" s="100" t="str">
+        <x:v>roster.003</x:v>
+      </x:c>
+      <x:c r="E1587" s="100" t="str">
+        <x:v>Owen Pike</x:v>
+      </x:c>
+      <x:c r="F1587" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1588" ht="30" customHeight="1">
+      <x:c r="A1588" s="95" t="str">
+        <x:v>ACT-002-roster.004</x:v>
+      </x:c>
+      <x:c r="B1588" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1588" s="95" t="str">
+        <x:v>Actual roster</x:v>
+      </x:c>
+      <x:c r="D1588" s="96" t="str">
+        <x:v>roster.004</x:v>
+      </x:c>
+      <x:c r="E1588" s="96" t="str">
+        <x:v>Dane Mercer (now named to Kip)</x:v>
+      </x:c>
+      <x:c r="F1588" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1589" ht="30" customHeight="1">
+      <x:c r="A1589" s="99" t="str">
+        <x:v>ACT-002-roster.005</x:v>
+      </x:c>
+      <x:c r="B1589" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1589" s="99" t="str">
+        <x:v>Actual roster</x:v>
+      </x:c>
+      <x:c r="D1589" s="100" t="str">
+        <x:v>roster.005</x:v>
+      </x:c>
+      <x:c r="E1589" s="100" t="str">
+        <x:v>Jory Hale</x:v>
+      </x:c>
+      <x:c r="F1589" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1590" ht="30" customHeight="1">
+      <x:c r="A1590" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Dominion Sight.rank</x:v>
+      </x:c>
+      <x:c r="B1590" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1590" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1590" s="96" t="str">
+        <x:v>abilities.Kip.Dominion Sight.rank</x:v>
+      </x:c>
+      <x:c r="E1590" s="96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1590" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1591" ht="30" customHeight="1">
+      <x:c r="A1591" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Dominion Sight.cost</x:v>
+      </x:c>
+      <x:c r="B1591" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1591" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1591" s="100" t="str">
+        <x:v>abilities.Kip.Dominion Sight.cost</x:v>
+      </x:c>
+      <x:c r="E1591" s="100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1591" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1592" ht="32" customHeight="1">
+      <x:c r="A1592" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Dominion Sight.inspection_seconds</x:v>
+      </x:c>
+      <x:c r="B1592" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1592" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1592" s="96" t="str">
+        <x:v>abilities.Kip.Dominion Sight.inspection_seconds</x:v>
+      </x:c>
+      <x:c r="E1592" s="96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1592" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1593" ht="32" customHeight="1">
+      <x:c r="A1593" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Dominion Sight.range_metres</x:v>
+      </x:c>
+      <x:c r="B1593" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1593" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1593" s="100" t="str">
+        <x:v>abilities.Kip.Dominion Sight.range_metres</x:v>
+      </x:c>
+      <x:c r="E1593" s="100" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1593" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1594" ht="30" customHeight="1">
+      <x:c r="A1594" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Dominion Sight.targets</x:v>
+      </x:c>
+      <x:c r="B1594" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1594" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1594" s="96" t="str">
+        <x:v>abilities.Kip.Dominion Sight.targets</x:v>
+      </x:c>
+      <x:c r="E1594" s="96" t="str">
+        <x:v>Visible dungeon fixtures and Claim anchors; not people, hidden objects or private panels.</x:v>
+      </x:c>
+      <x:c r="F1594" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1595" ht="30" customHeight="1">
+      <x:c r="A1595" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.rank</x:v>
+      </x:c>
+      <x:c r="B1595" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1595" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1595" s="100" t="str">
+        <x:v>abilities.Kip.Override.rank</x:v>
+      </x:c>
+      <x:c r="E1595" s="100" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1595" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1596" ht="30" customHeight="1">
+      <x:c r="A1596" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.cost</x:v>
+      </x:c>
+      <x:c r="B1596" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1596" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1596" s="96" t="str">
+        <x:v>abilities.Kip.Override.cost</x:v>
+      </x:c>
+      <x:c r="E1596" s="96" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1596" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1597" ht="30" customHeight="1">
+      <x:c r="A1597" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.range_metres</x:v>
+      </x:c>
+      <x:c r="B1597" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1597" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1597" s="100" t="str">
+        <x:v>abilities.Kip.Override.range_metres</x:v>
+      </x:c>
+      <x:c r="E1597" s="100" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1597" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1598" ht="32" customHeight="1">
+      <x:c r="A1598" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.duration_seconds</x:v>
+      </x:c>
+      <x:c r="B1598" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1598" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1598" s="96" t="str">
+        <x:v>abilities.Kip.Override.duration_seconds</x:v>
+      </x:c>
+      <x:c r="E1598" s="96" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F1598" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1599" ht="32" customHeight="1">
+      <x:c r="A1599" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.same_fixture_cooldown_after_control_seconds</x:v>
+      </x:c>
+      <x:c r="B1599" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1599" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1599" s="100" t="str">
+        <x:v>abilities.Kip.Override.same_fixture_cooldown_after_control_seconds</x:v>
+      </x:c>
+      <x:c r="E1599" s="100" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1599" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1600" ht="30" customHeight="1">
+      <x:c r="A1600" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.active_limit</x:v>
+      </x:c>
+      <x:c r="B1600" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1600" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1600" s="96" t="str">
+        <x:v>abilities.Kip.Override.active_limit</x:v>
+      </x:c>
+      <x:c r="E1600" s="96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1600" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1601" ht="32" customHeight="1">
+      <x:c r="A1601" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.limits</x:v>
+      </x:c>
+      <x:c r="B1601" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1601" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1601" s="100" t="str">
+        <x:v>abilities.Kip.Override.limits</x:v>
+      </x:c>
+      <x:c r="E1601" s="100" t="str">
+        <x:v>Available visible constructed defense; normal arc, fuel and reset. No creation, reload, repair or body control.</x:v>
+      </x:c>
+      <x:c r="F1601" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1602" ht="32" customHeight="1">
+      <x:c r="A1602" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Override.actual_use</x:v>
+      </x:c>
+      <x:c r="B1602" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1602" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1602" s="96" t="str">
+        <x:v>abilities.Kip.Override.actual_use</x:v>
+      </x:c>
+      <x:c r="E1602" s="96" t="str">
+        <x:v>Two paid uses since arrival: first launcher shot in Episode 1; second vent sweep in Episode 2. Both ended; no permanent fixture ownership.</x:v>
+      </x:c>
+      <x:c r="F1602" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1603" ht="30" customHeight="1">
+      <x:c r="A1603" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.rank</x:v>
+      </x:c>
+      <x:c r="B1603" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1603" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1603" s="100" t="str">
+        <x:v>abilities.Kip.Claim Room.rank</x:v>
+      </x:c>
+      <x:c r="E1603" s="100" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1603" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1604" ht="30" customHeight="1">
+      <x:c r="A1604" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.cost</x:v>
+      </x:c>
+      <x:c r="B1604" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1604" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1604" s="96" t="str">
+        <x:v>abilities.Kip.Claim Room.cost</x:v>
+      </x:c>
+      <x:c r="E1604" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1604" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1605" ht="30" customHeight="1">
+      <x:c r="A1605" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.touch_seconds</x:v>
+      </x:c>
+      <x:c r="B1605" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1605" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1605" s="100" t="str">
+        <x:v>abilities.Kip.Claim Room.touch_seconds</x:v>
+      </x:c>
+      <x:c r="E1605" s="100" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F1605" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1606" ht="32" customHeight="1">
+      <x:c r="A1606" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.room_max_metres</x:v>
+      </x:c>
+      <x:c r="B1606" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1606" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1606" s="96" t="str">
+        <x:v>abilities.Kip.Claim Room.room_max_metres</x:v>
+      </x:c>
+      <x:c r="E1606" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1606" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1607" ht="30" customHeight="1">
+      <x:c r="A1607" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.capacity</x:v>
+      </x:c>
+      <x:c r="B1607" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1607" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1607" s="100" t="str">
+        <x:v>abilities.Kip.Claim Room.capacity</x:v>
+      </x:c>
+      <x:c r="E1607" s="100" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1607" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1608" ht="32" customHeight="1">
+      <x:c r="A1608" s="95" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.limits</x:v>
+      </x:c>
+      <x:c r="B1608" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1608" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1608" s="96" t="str">
+        <x:v>abilities.Kip.Claim Room.limits</x:v>
+      </x:c>
+      <x:c r="E1608" s="96" t="str">
+        <x:v>Intact Claimable anchor; guardian defeated, seal absent, no living hostiles inside. Interruptions spend paid Mana. No automatic healing or barrier.</x:v>
+      </x:c>
+      <x:c r="F1608" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1609" ht="30" customHeight="1">
+      <x:c r="A1609" s="99" t="str">
+        <x:v>ACT-002-abilities.Kip.Claim Room.actual_use</x:v>
+      </x:c>
+      <x:c r="B1609" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1609" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1609" s="100" t="str">
+        <x:v>abilities.Kip.Claim Room.actual_use</x:v>
+      </x:c>
+      <x:c r="E1609" s="100" t="str">
+        <x:v>Available but unused.</x:v>
+      </x:c>
+      <x:c r="F1609" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1610" ht="30" customHeight="1">
+      <x:c r="A1610" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.rank</x:v>
+      </x:c>
+      <x:c r="B1610" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1610" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1610" s="96" t="str">
+        <x:v>abilities.Tessa.Quickstep.rank</x:v>
+      </x:c>
+      <x:c r="E1610" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1610" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1611" ht="30" customHeight="1">
+      <x:c r="A1611" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.cost</x:v>
+      </x:c>
+      <x:c r="B1611" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1611" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1611" s="100" t="str">
+        <x:v>abilities.Tessa.Quickstep.cost</x:v>
+      </x:c>
+      <x:c r="E1611" s="100" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1611" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1612" ht="32" customHeight="1">
+      <x:c r="A1612" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1612" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1612" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1612" s="96" t="str">
+        <x:v>abilities.Tessa.Quickstep.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1612" s="96" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1612" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1613" ht="32" customHeight="1">
+      <x:c r="A1613" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.distance_metres</x:v>
+      </x:c>
+      <x:c r="B1613" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1613" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1613" s="100" t="str">
+        <x:v>abilities.Tessa.Quickstep.distance_metres</x:v>
+      </x:c>
+      <x:c r="E1613" s="100" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F1613" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1614" ht="32" customHeight="1">
+      <x:c r="A1614" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.duration_seconds</x:v>
+      </x:c>
+      <x:c r="B1614" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1614" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1614" s="96" t="str">
+        <x:v>abilities.Tessa.Quickstep.duration_seconds</x:v>
+      </x:c>
+      <x:c r="E1614" s="96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1614" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1615" ht="30" customHeight="1">
+      <x:c r="A1615" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.limits</x:v>
+      </x:c>
+      <x:c r="B1615" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1615" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1615" s="100" t="str">
+        <x:v>abilities.Tessa.Quickstep.limits</x:v>
+      </x:c>
+      <x:c r="E1615" s="100" t="str">
+        <x:v>Traversable physical route; no teleport, impossible gap or carrying another adult.</x:v>
+      </x:c>
+      <x:c r="F1615" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1616" ht="30" customHeight="1">
+      <x:c r="A1616" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Quickstep.actual_use</x:v>
+      </x:c>
+      <x:c r="B1616" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1616" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1616" s="96" t="str">
+        <x:v>abilities.Tessa.Quickstep.actual_use</x:v>
+      </x:c>
+      <x:c r="E1616" s="96" t="str">
+        <x:v>One paid use after Kip arrives.</x:v>
+      </x:c>
+      <x:c r="F1616" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1617" ht="30" customHeight="1">
+      <x:c r="A1617" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.rank</x:v>
+      </x:c>
+      <x:c r="B1617" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1617" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1617" s="100" t="str">
+        <x:v>abilities.Tessa.Trail Sight.rank</x:v>
+      </x:c>
+      <x:c r="E1617" s="100" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1617" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1618" ht="30" customHeight="1">
+      <x:c r="A1618" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.cost</x:v>
+      </x:c>
+      <x:c r="B1618" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1618" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1618" s="96" t="str">
+        <x:v>abilities.Tessa.Trail Sight.cost</x:v>
+      </x:c>
+      <x:c r="E1618" s="96" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1618" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1619" ht="32" customHeight="1">
+      <x:c r="A1619" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1619" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1619" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1619" s="100" t="str">
+        <x:v>abilities.Tessa.Trail Sight.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1619" s="100" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F1619" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1620" ht="32" customHeight="1">
+      <x:c r="A1620" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.duration_seconds</x:v>
+      </x:c>
+      <x:c r="B1620" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1620" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1620" s="96" t="str">
+        <x:v>abilities.Tessa.Trail Sight.duration_seconds</x:v>
+      </x:c>
+      <x:c r="E1620" s="96" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F1620" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1621" ht="32" customHeight="1">
+      <x:c r="A1621" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.range_metres</x:v>
+      </x:c>
+      <x:c r="B1621" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1621" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1621" s="100" t="str">
+        <x:v>abilities.Tessa.Trail Sight.range_metres</x:v>
+      </x:c>
+      <x:c r="E1621" s="100" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F1621" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1622" ht="32" customHeight="1">
+      <x:c r="A1622" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.track_age_max_hours</x:v>
+      </x:c>
+      <x:c r="B1622" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1622" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1622" s="96" t="str">
+        <x:v>abilities.Tessa.Trail Sight.track_age_max_hours</x:v>
+      </x:c>
+      <x:c r="E1622" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1622" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1623" ht="30" customHeight="1">
+      <x:c r="A1623" s="99" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.limits</x:v>
+      </x:c>
+      <x:c r="B1623" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1623" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1623" s="100" t="str">
+        <x:v>abilities.Tessa.Trail Sight.limits</x:v>
+      </x:c>
+      <x:c r="E1623" s="100" t="str">
+        <x:v>Visible surviving traces from inspected source; no live location, thoughts or walls.</x:v>
+      </x:c>
+      <x:c r="F1623" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1624" ht="30" customHeight="1">
+      <x:c r="A1624" s="95" t="str">
+        <x:v>ACT-002-abilities.Tessa.Trail Sight.actual_use</x:v>
+      </x:c>
+      <x:c r="B1624" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1624" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1624" s="96" t="str">
+        <x:v>abilities.Tessa.Trail Sight.actual_use</x:v>
+      </x:c>
+      <x:c r="E1624" s="96" t="str">
+        <x:v>Not used after Kip arrives.</x:v>
+      </x:c>
+      <x:c r="F1624" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1625" ht="30" customHeight="1">
+      <x:c r="A1625" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.rank</x:v>
+      </x:c>
+      <x:c r="B1625" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1625" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1625" s="100" t="str">
+        <x:v>abilities.Owen.Staunch.rank</x:v>
+      </x:c>
+      <x:c r="E1625" s="100" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1625" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1626" ht="30" customHeight="1">
+      <x:c r="A1626" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.cost</x:v>
+      </x:c>
+      <x:c r="B1626" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1626" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1626" s="96" t="str">
+        <x:v>abilities.Owen.Staunch.cost</x:v>
+      </x:c>
+      <x:c r="E1626" s="96" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1626" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1627" ht="32" customHeight="1">
+      <x:c r="A1627" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1627" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1627" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1627" s="100" t="str">
+        <x:v>abilities.Owen.Staunch.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1627" s="100" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1627" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1628" ht="30" customHeight="1">
+      <x:c r="A1628" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.touch_seconds</x:v>
+      </x:c>
+      <x:c r="B1628" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1628" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1628" s="96" t="str">
+        <x:v>abilities.Owen.Staunch.touch_seconds</x:v>
+      </x:c>
+      <x:c r="E1628" s="96" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F1628" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1629" ht="30" customHeight="1">
+      <x:c r="A1629" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.seal_minutes</x:v>
+      </x:c>
+      <x:c r="B1629" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1629" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1629" s="100" t="str">
+        <x:v>abilities.Owen.Staunch.seal_minutes</x:v>
+      </x:c>
+      <x:c r="E1629" s="100" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F1629" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1630" ht="30" customHeight="1">
+      <x:c r="A1630" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Staunch.limits</x:v>
+      </x:c>
+      <x:c r="B1630" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1630" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1630" s="96" t="str">
+        <x:v>abilities.Owen.Staunch.limits</x:v>
+      </x:c>
+      <x:c r="E1630" s="96" t="str">
+        <x:v>One external wound; no blood replacement, internal healing or revival; strain or blow can break seal.</x:v>
+      </x:c>
+      <x:c r="F1630" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1631" ht="30" customHeight="1">
+      <x:c r="A1631" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.rank</x:v>
+      </x:c>
+      <x:c r="B1631" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1631" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1631" s="100" t="str">
+        <x:v>abilities.Owen.Mend.rank</x:v>
+      </x:c>
+      <x:c r="E1631" s="100" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1631" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1632" ht="30" customHeight="1">
+      <x:c r="A1632" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.cost</x:v>
+      </x:c>
+      <x:c r="B1632" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1632" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1632" s="96" t="str">
+        <x:v>abilities.Owen.Mend.cost</x:v>
+      </x:c>
+      <x:c r="E1632" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1632" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1633" ht="30" customHeight="1">
+      <x:c r="A1633" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1633" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1633" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1633" s="100" t="str">
+        <x:v>abilities.Owen.Mend.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1633" s="100" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F1633" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1634" ht="30" customHeight="1">
+      <x:c r="A1634" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.touch_seconds</x:v>
+      </x:c>
+      <x:c r="B1634" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1634" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1634" s="96" t="str">
+        <x:v>abilities.Owen.Mend.touch_seconds</x:v>
+      </x:c>
+      <x:c r="E1634" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1634" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1635" ht="32" customHeight="1">
+      <x:c r="A1635" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.wound_max_length_cm</x:v>
+      </x:c>
+      <x:c r="B1635" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1635" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1635" s="100" t="str">
+        <x:v>abilities.Owen.Mend.wound_max_length_cm</x:v>
+      </x:c>
+      <x:c r="E1635" s="100" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1635" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1636" ht="30" customHeight="1">
+      <x:c r="A1636" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.wound_max_depth_cm</x:v>
+      </x:c>
+      <x:c r="B1636" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1636" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1636" s="96" t="str">
+        <x:v>abilities.Owen.Mend.wound_max_depth_cm</x:v>
+      </x:c>
+      <x:c r="E1636" s="96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F1636" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1637" ht="30" customHeight="1">
+      <x:c r="A1637" s="99" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.limits</x:v>
+      </x:c>
+      <x:c r="B1637" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1637" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1637" s="100" t="str">
+        <x:v>abilities.Owen.Mend.limits</x:v>
+      </x:c>
+      <x:c r="E1637" s="100" t="str">
+        <x:v>Aligned present skin and shallow muscle; no bone, organs, major vessels, nerves, regrowth or lost blood.</x:v>
+      </x:c>
+      <x:c r="F1637" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1638" ht="30" customHeight="1">
+      <x:c r="A1638" s="95" t="str">
+        <x:v>ACT-002-abilities.Owen.Mend.actual_use</x:v>
+      </x:c>
+      <x:c r="B1638" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1638" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1638" s="96" t="str">
+        <x:v>abilities.Owen.Mend.actual_use</x:v>
+      </x:c>
+      <x:c r="E1638" s="96" t="str">
+        <x:v>One full twenty-second cast after arrival, closing Kip's shallow forearm cut. Jory's fracture remains.</x:v>
+      </x:c>
+      <x:c r="F1638" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1639" ht="30" customHeight="1">
+      <x:c r="A1639" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.rank</x:v>
+      </x:c>
+      <x:c r="B1639" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1639" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1639" s="100" t="str">
+        <x:v>abilities.Dane.Interpose.rank</x:v>
+      </x:c>
+      <x:c r="E1639" s="100" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1639" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1640" ht="30" customHeight="1">
+      <x:c r="A1640" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.cost</x:v>
+      </x:c>
+      <x:c r="B1640" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1640" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1640" s="96" t="str">
+        <x:v>abilities.Dane.Interpose.cost</x:v>
+      </x:c>
+      <x:c r="E1640" s="96" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1640" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1641" ht="32" customHeight="1">
+      <x:c r="A1641" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1641" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1641" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1641" s="100" t="str">
+        <x:v>abilities.Dane.Interpose.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1641" s="100" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1641" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1642" ht="32" customHeight="1">
+      <x:c r="A1642" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.distance_metres</x:v>
+      </x:c>
+      <x:c r="B1642" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1642" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1642" s="96" t="str">
+        <x:v>abilities.Dane.Interpose.distance_metres</x:v>
+      </x:c>
+      <x:c r="E1642" s="96" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F1642" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1643" ht="32" customHeight="1">
+      <x:c r="A1643" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.block_window_seconds</x:v>
+      </x:c>
+      <x:c r="B1643" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1643" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1643" s="100" t="str">
+        <x:v>abilities.Dane.Interpose.block_window_seconds</x:v>
+      </x:c>
+      <x:c r="E1643" s="100" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F1643" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1644" ht="32" customHeight="1">
+      <x:c r="A1644" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.block_strength_multiplier</x:v>
+      </x:c>
+      <x:c r="B1644" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1644" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1644" s="96" t="str">
+        <x:v>abilities.Dane.Interpose.block_strength_multiplier</x:v>
+      </x:c>
+      <x:c r="E1644" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1644" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1645" ht="30" customHeight="1">
+      <x:c r="A1645" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Interpose.limits</x:v>
+      </x:c>
+      <x:c r="B1645" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1645" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1645" s="100" t="str">
+        <x:v>abilities.Dane.Interpose.limits</x:v>
+      </x:c>
+      <x:c r="E1645" s="100" t="str">
+        <x:v>Clear physical path to visible ally/threat; next deliberate block, not stronger bones or teleport.</x:v>
+      </x:c>
+      <x:c r="F1645" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1646" ht="30" customHeight="1">
+      <x:c r="A1646" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.rank</x:v>
+      </x:c>
+      <x:c r="B1646" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1646" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1646" s="96" t="str">
+        <x:v>abilities.Dane.Bulwark.rank</x:v>
+      </x:c>
+      <x:c r="E1646" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1646" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1647" ht="30" customHeight="1">
+      <x:c r="A1647" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.cost</x:v>
+      </x:c>
+      <x:c r="B1647" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1647" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1647" s="100" t="str">
+        <x:v>abilities.Dane.Bulwark.cost</x:v>
+      </x:c>
+      <x:c r="E1647" s="100" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1647" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1648" ht="32" customHeight="1">
+      <x:c r="A1648" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="B1648" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1648" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1648" s="96" t="str">
+        <x:v>abilities.Dane.Bulwark.cooldown_seconds</x:v>
+      </x:c>
+      <x:c r="E1648" s="96" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F1648" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1649" ht="32" customHeight="1">
+      <x:c r="A1649" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.duration_seconds</x:v>
+      </x:c>
+      <x:c r="B1649" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1649" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1649" s="100" t="str">
+        <x:v>abilities.Dane.Bulwark.duration_seconds</x:v>
+      </x:c>
+      <x:c r="E1649" s="100" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F1649" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1650" ht="32" customHeight="1">
+      <x:c r="A1650" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.front_width_metres</x:v>
+      </x:c>
+      <x:c r="B1650" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1650" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1650" s="96" t="str">
+        <x:v>abilities.Dane.Bulwark.front_width_metres</x:v>
+      </x:c>
+      <x:c r="E1650" s="96" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F1650" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1651" ht="32" customHeight="1">
+      <x:c r="A1651" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.front_height_metres</x:v>
+      </x:c>
+      <x:c r="B1651" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1651" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1651" s="100" t="str">
+        <x:v>abilities.Dane.Bulwark.front_height_metres</x:v>
+      </x:c>
+      <x:c r="E1651" s="100" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1651" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1652" ht="32" customHeight="1">
+      <x:c r="A1652" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.physical_force_multiplier</x:v>
+      </x:c>
+      <x:c r="B1652" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1652" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1652" s="96" t="str">
+        <x:v>abilities.Dane.Bulwark.physical_force_multiplier</x:v>
+      </x:c>
+      <x:c r="E1652" s="96" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F1652" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1653" ht="32" customHeight="1">
+      <x:c r="A1653" s="99" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.limits</x:v>
+      </x:c>
+      <x:c r="B1653" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1653" s="99" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1653" s="100" t="str">
+        <x:v>abilities.Dane.Bulwark.limits</x:v>
+      </x:c>
+      <x:c r="E1653" s="100" t="str">
+        <x:v>Raised weapon, concentration and facing; no heat, poison or rear protection. Mutually exclusive with own Interpose.</x:v>
+      </x:c>
+      <x:c r="F1653" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1654" ht="32" customHeight="1">
+      <x:c r="A1654" s="95" t="str">
+        <x:v>ACT-002-abilities.Dane.Bulwark.actual_use</x:v>
+      </x:c>
+      <x:c r="B1654" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1654" s="95" t="str">
+        <x:v>Actual abilities</x:v>
+      </x:c>
+      <x:c r="D1654" s="96" t="str">
+        <x:v>abilities.Dane.Bulwark.actual_use</x:v>
+      </x:c>
+      <x:c r="E1654" s="96" t="str">
+        <x:v>One paid eight-second defense in Episode 2 while retreating at a walk; effect ended before Kip fired the vent.</x:v>
+      </x:c>
+      <x:c r="F1654" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1655" ht="30" customHeight="1">
+      <x:c r="A1655" s="99" t="str">
+        <x:v>ACT-002-owned_rooms.Kip</x:v>
+      </x:c>
+      <x:c r="B1655" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1655" s="99" t="str">
+        <x:v>Actual owned_rooms</x:v>
+      </x:c>
+      <x:c r="D1655" s="100" t="str">
+        <x:v>owned_rooms.Kip</x:v>
+      </x:c>
+      <x:c r="E1655" s="100" t="str">
+        <x:v>None recorded</x:v>
+      </x:c>
+      <x:c r="F1655" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1656" ht="30" customHeight="1">
+      <x:c r="A1656" s="95" t="str">
+        <x:v>ACT-002-owned_rooms.Tessa</x:v>
+      </x:c>
+      <x:c r="B1656" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1656" s="95" t="str">
+        <x:v>Actual owned_rooms</x:v>
+      </x:c>
+      <x:c r="D1656" s="96" t="str">
+        <x:v>owned_rooms.Tessa</x:v>
+      </x:c>
+      <x:c r="E1656" s="96" t="str">
+        <x:v>None recorded</x:v>
+      </x:c>
+      <x:c r="F1656" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1657" ht="30" customHeight="1">
+      <x:c r="A1657" s="99" t="str">
+        <x:v>ACT-002-owned_rooms.Owen</x:v>
+      </x:c>
+      <x:c r="B1657" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1657" s="99" t="str">
+        <x:v>Actual owned_rooms</x:v>
+      </x:c>
+      <x:c r="D1657" s="100" t="str">
+        <x:v>owned_rooms.Owen</x:v>
+      </x:c>
+      <x:c r="E1657" s="100" t="str">
+        <x:v>None recorded</x:v>
+      </x:c>
+      <x:c r="F1657" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1658" ht="30" customHeight="1">
+      <x:c r="A1658" s="95" t="str">
+        <x:v>ACT-002-owned_rooms.Dane</x:v>
+      </x:c>
+      <x:c r="B1658" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1658" s="95" t="str">
+        <x:v>Actual owned_rooms</x:v>
+      </x:c>
+      <x:c r="D1658" s="96" t="str">
+        <x:v>owned_rooms.Dane</x:v>
+      </x:c>
+      <x:c r="E1658" s="96" t="str">
+        <x:v>None recorded</x:v>
+      </x:c>
+      <x:c r="F1658" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1659" ht="30" customHeight="1">
+      <x:c r="A1659" s="99" t="str">
+        <x:v>ACT-002-fatigue.Kip</x:v>
+      </x:c>
+      <x:c r="B1659" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1659" s="99" t="str">
+        <x:v>Actual fatigue</x:v>
+      </x:c>
+      <x:c r="D1659" s="100" t="str">
+        <x:v>fatigue.Kip</x:v>
+      </x:c>
+      <x:c r="E1659" s="100" t="str">
+        <x:v>Alert but shoulders still ache and fingers cramped from carrying; leveling did not remove fatigue.</x:v>
+      </x:c>
+      <x:c r="F1659" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1660" ht="30" customHeight="1">
+      <x:c r="A1660" s="95" t="str">
+        <x:v>ACT-002-fatigue.companions</x:v>
+      </x:c>
+      <x:c r="B1660" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1660" s="95" t="str">
+        <x:v>Actual fatigue</x:v>
+      </x:c>
+      <x:c r="D1660" s="96" t="str">
+        <x:v>fatigue.companions</x:v>
+      </x:c>
+      <x:c r="E1660" s="96" t="str">
+        <x:v>Still alert and actively checking/caring for the group. No sleep or eligible Mana recovery credited.</x:v>
+      </x:c>
+      <x:c r="F1660" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1661" ht="32" customHeight="1">
+      <x:c r="A1661" s="99" t="str">
+        <x:v>ACT-002-relationships.Kip and Dane</x:v>
+      </x:c>
+      <x:c r="B1661" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1661" s="99" t="str">
+        <x:v>Actual relationships</x:v>
+      </x:c>
+      <x:c r="D1661" s="100" t="str">
+        <x:v>relationships.Kip and Dane</x:v>
+      </x:c>
+      <x:c r="E1661" s="100" t="str">
+        <x:v>Dane accepts a specific limited plan, credits Kip for the escape and asks him to admit uncertainty before making broad promises. Kip accepts the correction.</x:v>
+      </x:c>
+      <x:c r="F1661" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1662" ht="32" customHeight="1">
+      <x:c r="A1662" s="95" t="str">
+        <x:v>ACT-002-relationships.Kip and Owen</x:v>
+      </x:c>
+      <x:c r="B1662" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1662" s="95" t="str">
+        <x:v>Actual relationships</x:v>
+      </x:c>
+      <x:c r="D1662" s="96" t="str">
+        <x:v>relationships.Kip and Owen</x:v>
+      </x:c>
+      <x:c r="E1662" s="96" t="str">
+        <x:v>Kip initially puts Jory first; Owen explains the treatable cut versus the persistent fracture and accepts thanks through practical help.</x:v>
+      </x:c>
+      <x:c r="F1662" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1663" ht="32" customHeight="1">
+      <x:c r="A1663" s="99" t="str">
+        <x:v>ACT-002-relationships.Kip and group</x:v>
+      </x:c>
+      <x:c r="B1663" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1663" s="99" t="str">
+        <x:v>Actual relationships</x:v>
+      </x:c>
+      <x:c r="D1663" s="100" t="str">
+        <x:v>relationships.Kip and group</x:v>
+      </x:c>
+      <x:c r="E1663" s="100" t="str">
+        <x:v>Cooperation strengthened through the retreat and aftercare; private origin, legendary class and deep trust remain unshared.</x:v>
+      </x:c>
+      <x:c r="F1663" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1664" ht="30" customHeight="1">
+      <x:c r="A1664" s="95" t="str">
+        <x:v>ACT-002-unresolved_threats.001</x:v>
+      </x:c>
+      <x:c r="B1664" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1664" s="95" t="str">
+        <x:v>Actual unresolved_threats</x:v>
+      </x:c>
+      <x:c r="D1664" s="96" t="str">
+        <x:v>unresolved_threats.001</x:v>
+      </x:c>
+      <x:c r="E1664" s="96" t="str">
+        <x:v>The wounded hunter may return; its current location is unknown after its scraping faded.</x:v>
+      </x:c>
+      <x:c r="F1664" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1665" ht="32" customHeight="1">
+      <x:c r="A1665" s="99" t="str">
+        <x:v>ACT-002-unresolved_threats.002</x:v>
+      </x:c>
+      <x:c r="B1665" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1665" s="99" t="str">
+        <x:v>Actual unresolved_threats</x:v>
+      </x:c>
+      <x:c r="D1665" s="100" t="str">
+        <x:v>unresolved_threats.002</x:v>
+      </x:c>
+      <x:c r="E1665" s="100" t="str">
+        <x:v>The chamber is not claimed, the route onward is physically obstructed, and escape from Cinderwell remains unresolved.</x:v>
+      </x:c>
+      <x:c r="F1665" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1666" ht="30" customHeight="1">
+      <x:c r="A1666" s="95" t="str">
+        <x:v>ACT-002-unresolved_threats.003</x:v>
+      </x:c>
+      <x:c r="B1666" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1666" s="95" t="str">
+        <x:v>Actual unresolved_threats</x:v>
+      </x:c>
+      <x:c r="D1666" s="96" t="str">
+        <x:v>unresolved_threats.003</x:v>
+      </x:c>
+      <x:c r="E1666" s="96" t="str">
+        <x:v>Kip must learn Claim Room's actual terms and evaluate the anchor before a valid activation.</x:v>
+      </x:c>
+      <x:c r="F1666" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1667" ht="30" customHeight="1">
+      <x:c r="A1667" s="99" t="str">
+        <x:v>ACT-002-resource_events.001.person</x:v>
+      </x:c>
+      <x:c r="B1667" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1667" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1667" s="100" t="str">
+        <x:v>resource_events.001.person</x:v>
+      </x:c>
+      <x:c r="E1667" s="100" t="str">
+        <x:v>Dane</x:v>
+      </x:c>
+      <x:c r="F1667" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1668" ht="30" customHeight="1">
+      <x:c r="A1668" s="95" t="str">
+        <x:v>ACT-002-resource_events.001.event</x:v>
+      </x:c>
+      <x:c r="B1668" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1668" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1668" s="96" t="str">
+        <x:v>resource_events.001.event</x:v>
+      </x:c>
+      <x:c r="E1668" s="96" t="str">
+        <x:v>Bulwark during protected litter retreat</x:v>
+      </x:c>
+      <x:c r="F1668" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1669" ht="30" customHeight="1">
+      <x:c r="A1669" s="99" t="str">
+        <x:v>ACT-002-resource_events.001.before</x:v>
+      </x:c>
+      <x:c r="B1669" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1669" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1669" s="100" t="str">
+        <x:v>resource_events.001.before</x:v>
+      </x:c>
+      <x:c r="E1669" s="100" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F1669" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1670" ht="30" customHeight="1">
+      <x:c r="A1670" s="95" t="str">
+        <x:v>ACT-002-resource_events.001.cost</x:v>
+      </x:c>
+      <x:c r="B1670" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1670" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1670" s="96" t="str">
+        <x:v>resource_events.001.cost</x:v>
+      </x:c>
+      <x:c r="E1670" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1670" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1671" ht="30" customHeight="1">
+      <x:c r="A1671" s="99" t="str">
+        <x:v>ACT-002-resource_events.001.recovery</x:v>
+      </x:c>
+      <x:c r="B1671" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1671" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1671" s="100" t="str">
+        <x:v>resource_events.001.recovery</x:v>
+      </x:c>
+      <x:c r="E1671" s="100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1671" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1672" ht="30" customHeight="1">
+      <x:c r="A1672" s="95" t="str">
+        <x:v>ACT-002-resource_events.001.after</x:v>
+      </x:c>
+      <x:c r="B1672" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1672" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1672" s="96" t="str">
+        <x:v>resource_events.001.after</x:v>
+      </x:c>
+      <x:c r="E1672" s="96" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F1672" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1673" ht="30" customHeight="1">
+      <x:c r="A1673" s="99" t="str">
+        <x:v>ACT-002-resource_events.001.maximum</x:v>
+      </x:c>
+      <x:c r="B1673" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1673" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1673" s="100" t="str">
+        <x:v>resource_events.001.maximum</x:v>
+      </x:c>
+      <x:c r="E1673" s="100" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F1673" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1674" ht="30" customHeight="1">
+      <x:c r="A1674" s="95" t="str">
+        <x:v>ACT-002-resource_events.002.person</x:v>
+      </x:c>
+      <x:c r="B1674" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1674" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1674" s="96" t="str">
+        <x:v>resource_events.002.person</x:v>
+      </x:c>
+      <x:c r="E1674" s="96" t="str">
+        <x:v>Kip</x:v>
+      </x:c>
+      <x:c r="F1674" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1675" ht="30" customHeight="1">
+      <x:c r="A1675" s="99" t="str">
+        <x:v>ACT-002-resource_events.002.event</x:v>
+      </x:c>
+      <x:c r="B1675" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1675" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1675" s="100" t="str">
+        <x:v>resource_events.002.event</x:v>
+      </x:c>
+      <x:c r="E1675" s="100" t="str">
+        <x:v>Second Override: full five-second fire vent sweep</x:v>
+      </x:c>
+      <x:c r="F1675" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1676" ht="30" customHeight="1">
+      <x:c r="A1676" s="95" t="str">
+        <x:v>ACT-002-resource_events.002.before</x:v>
+      </x:c>
+      <x:c r="B1676" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1676" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1676" s="96" t="str">
+        <x:v>resource_events.002.before</x:v>
+      </x:c>
+      <x:c r="E1676" s="96" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F1676" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1677" ht="30" customHeight="1">
+      <x:c r="A1677" s="99" t="str">
+        <x:v>ACT-002-resource_events.002.cost</x:v>
+      </x:c>
+      <x:c r="B1677" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1677" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1677" s="100" t="str">
+        <x:v>resource_events.002.cost</x:v>
+      </x:c>
+      <x:c r="E1677" s="100" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1677" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1678" ht="30" customHeight="1">
+      <x:c r="A1678" s="95" t="str">
+        <x:v>ACT-002-resource_events.002.recovery</x:v>
+      </x:c>
+      <x:c r="B1678" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1678" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1678" s="96" t="str">
+        <x:v>resource_events.002.recovery</x:v>
+      </x:c>
+      <x:c r="E1678" s="96" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1678" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1679" ht="30" customHeight="1">
+      <x:c r="A1679" s="99" t="str">
+        <x:v>ACT-002-resource_events.002.after</x:v>
+      </x:c>
+      <x:c r="B1679" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1679" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1679" s="100" t="str">
+        <x:v>resource_events.002.after</x:v>
+      </x:c>
+      <x:c r="E1679" s="100" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1679" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1680" ht="30" customHeight="1">
+      <x:c r="A1680" s="95" t="str">
+        <x:v>ACT-002-resource_events.002.maximum</x:v>
+      </x:c>
+      <x:c r="B1680" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1680" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1680" s="96" t="str">
+        <x:v>resource_events.002.maximum</x:v>
+      </x:c>
+      <x:c r="E1680" s="96" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F1680" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1681" ht="30" customHeight="1">
+      <x:c r="A1681" s="99" t="str">
+        <x:v>ACT-002-resource_events.003.person</x:v>
+      </x:c>
+      <x:c r="B1681" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1681" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1681" s="100" t="str">
+        <x:v>resource_events.003.person</x:v>
+      </x:c>
+      <x:c r="E1681" s="100" t="str">
+        <x:v>Owen</x:v>
+      </x:c>
+      <x:c r="F1681" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1682" ht="30" customHeight="1">
+      <x:c r="A1682" s="95" t="str">
+        <x:v>ACT-002-resource_events.003.event</x:v>
+      </x:c>
+      <x:c r="B1682" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1682" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1682" s="96" t="str">
+        <x:v>resource_events.003.event</x:v>
+      </x:c>
+      <x:c r="E1682" s="96" t="str">
+        <x:v>One full Mend on Kip forearm</x:v>
+      </x:c>
+      <x:c r="F1682" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1683" ht="30" customHeight="1">
+      <x:c r="A1683" s="99" t="str">
+        <x:v>ACT-002-resource_events.003.before</x:v>
+      </x:c>
+      <x:c r="B1683" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1683" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1683" s="100" t="str">
+        <x:v>resource_events.003.before</x:v>
+      </x:c>
+      <x:c r="E1683" s="100" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F1683" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1684" ht="30" customHeight="1">
+      <x:c r="A1684" s="95" t="str">
+        <x:v>ACT-002-resource_events.003.cost</x:v>
+      </x:c>
+      <x:c r="B1684" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1684" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1684" s="96" t="str">
+        <x:v>resource_events.003.cost</x:v>
+      </x:c>
+      <x:c r="E1684" s="96" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1684" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1685" ht="30" customHeight="1">
+      <x:c r="A1685" s="99" t="str">
+        <x:v>ACT-002-resource_events.003.recovery</x:v>
+      </x:c>
+      <x:c r="B1685" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1685" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1685" s="100" t="str">
+        <x:v>resource_events.003.recovery</x:v>
+      </x:c>
+      <x:c r="E1685" s="100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1685" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1686" ht="30" customHeight="1">
+      <x:c r="A1686" s="95" t="str">
+        <x:v>ACT-002-resource_events.003.after</x:v>
+      </x:c>
+      <x:c r="B1686" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1686" s="95" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1686" s="96" t="str">
+        <x:v>resource_events.003.after</x:v>
+      </x:c>
+      <x:c r="E1686" s="96" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F1686" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1687" ht="30" customHeight="1">
+      <x:c r="A1687" s="99" t="str">
+        <x:v>ACT-002-resource_events.003.maximum</x:v>
+      </x:c>
+      <x:c r="B1687" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1687" s="99" t="str">
+        <x:v>Actual resource_events</x:v>
+      </x:c>
+      <x:c r="D1687" s="100" t="str">
+        <x:v>resource_events.003.maximum</x:v>
+      </x:c>
+      <x:c r="E1687" s="100" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F1687" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1688" ht="30" customHeight="1">
+      <x:c r="A1688" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.id</x:v>
+      </x:c>
+      <x:c r="B1688" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1688" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1688" s="96" t="str">
+        <x:v>xp_events.001.id</x:v>
+      </x:c>
+      <x:c r="E1688" s="96" t="str">
+        <x:v>retreat-001</x:v>
+      </x:c>
+      <x:c r="F1688" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1689" ht="30" customHeight="1">
+      <x:c r="A1689" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.rating</x:v>
+      </x:c>
+      <x:c r="B1689" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1689" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1689" s="100" t="str">
+        <x:v>xp_events.001.rating</x:v>
+      </x:c>
+      <x:c r="E1689" s="100" t="str">
+        <x:v>significant</x:v>
+      </x:c>
+      <x:c r="F1689" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1690" ht="32" customHeight="1">
+      <x:c r="A1690" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.award_per_eligible_person</x:v>
+      </x:c>
+      <x:c r="B1690" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1690" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1690" s="96" t="str">
+        <x:v>xp_events.001.award_per_eligible_person</x:v>
+      </x:c>
+      <x:c r="E1690" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F1690" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1691" ht="30" customHeight="1">
+      <x:c r="A1691" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.completed_after</x:v>
+      </x:c>
+      <x:c r="B1691" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1691" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1691" s="100" t="str">
+        <x:v>xp_events.001.completed_after</x:v>
+      </x:c>
+      <x:c r="E1691" s="100" t="str">
+        <x:v>Litter safe inside, injury aftercare completed, entrances checked</x:v>
+      </x:c>
+      <x:c r="F1691" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1692" ht="30" customHeight="1">
+      <x:c r="A1692" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.contributors.Kip</x:v>
+      </x:c>
+      <x:c r="B1692" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1692" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1692" s="96" t="str">
+        <x:v>xp_events.001.contributors.Kip</x:v>
+      </x:c>
+      <x:c r="E1692" s="96" t="str">
+        <x:v>Carried litter and redirected two existing defenses.</x:v>
+      </x:c>
+      <x:c r="F1692" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1693" ht="30" customHeight="1">
+      <x:c r="A1693" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.contributors.Tessa</x:v>
+      </x:c>
+      <x:c r="B1693" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1693" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1693" s="100" t="str">
+        <x:v>xp_events.001.contributors.Tessa</x:v>
+      </x:c>
+      <x:c r="E1693" s="100" t="str">
+        <x:v>Scouted crossing/route, helped close door and checked chamber.</x:v>
+      </x:c>
+      <x:c r="F1693" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1694" ht="30" customHeight="1">
+      <x:c r="A1694" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.contributors.Owen</x:v>
+      </x:c>
+      <x:c r="B1694" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1694" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1694" s="96" t="str">
+        <x:v>xp_events.001.contributors.Owen</x:v>
+      </x:c>
+      <x:c r="E1694" s="96" t="str">
+        <x:v>Carried litter and performed necessary aftercare.</x:v>
+      </x:c>
+      <x:c r="F1694" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1695" ht="30" customHeight="1">
+      <x:c r="A1695" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.contributors.Dane</x:v>
+      </x:c>
+      <x:c r="B1695" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1695" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1695" s="100" t="str">
+        <x:v>xp_events.001.contributors.Dane</x:v>
+      </x:c>
+      <x:c r="E1695" s="100" t="str">
+        <x:v>Held rearguard, protected movement, helped bar entrance and checked chamber.</x:v>
+      </x:c>
+      <x:c r="F1695" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1696" ht="30" customHeight="1">
+      <x:c r="A1696" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Kip.level</x:v>
+      </x:c>
+      <x:c r="B1696" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1696" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1696" s="96" t="str">
+        <x:v>xp_events.001.results.Kip.level</x:v>
+      </x:c>
+      <x:c r="E1696" s="96" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F1696" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1697" ht="30" customHeight="1">
+      <x:c r="A1697" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Kip.mana_current</x:v>
+      </x:c>
+      <x:c r="B1697" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1697" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1697" s="100" t="str">
+        <x:v>xp_events.001.results.Kip.mana_current</x:v>
+      </x:c>
+      <x:c r="E1697" s="100" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F1697" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1698" ht="30" customHeight="1">
+      <x:c r="A1698" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Kip.mana_max</x:v>
+      </x:c>
+      <x:c r="B1698" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1698" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1698" s="96" t="str">
+        <x:v>xp_events.001.results.Kip.mana_max</x:v>
+      </x:c>
+      <x:c r="E1698" s="96" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F1698" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1699" ht="30" customHeight="1">
+      <x:c r="A1699" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Kip.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="B1699" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1699" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1699" s="100" t="str">
+        <x:v>xp_events.001.results.Kip.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="E1699" s="100" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F1699" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1700" ht="30" customHeight="1">
+      <x:c r="A1700" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Kip.xp_to_next</x:v>
+      </x:c>
+      <x:c r="B1700" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1700" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1700" s="96" t="str">
+        <x:v>xp_events.001.results.Kip.xp_to_next</x:v>
+      </x:c>
+      <x:c r="E1700" s="96" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F1700" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1701" ht="30" customHeight="1">
+      <x:c r="A1701" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Tessa.level</x:v>
+      </x:c>
+      <x:c r="B1701" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1701" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1701" s="100" t="str">
+        <x:v>xp_events.001.results.Tessa.level</x:v>
+      </x:c>
+      <x:c r="E1701" s="100" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F1701" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1702" ht="32" customHeight="1">
+      <x:c r="A1702" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Tessa.mana_current</x:v>
+      </x:c>
+      <x:c r="B1702" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1702" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1702" s="96" t="str">
+        <x:v>xp_events.001.results.Tessa.mana_current</x:v>
+      </x:c>
+      <x:c r="E1702" s="96" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F1702" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1703" ht="30" customHeight="1">
+      <x:c r="A1703" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Tessa.mana_max</x:v>
+      </x:c>
+      <x:c r="B1703" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1703" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1703" s="100" t="str">
+        <x:v>xp_events.001.results.Tessa.mana_max</x:v>
+      </x:c>
+      <x:c r="E1703" s="100" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F1703" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1704" ht="30" customHeight="1">
+      <x:c r="A1704" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Tessa.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="B1704" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1704" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1704" s="96" t="str">
+        <x:v>xp_events.001.results.Tessa.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="E1704" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F1704" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1705" ht="30" customHeight="1">
+      <x:c r="A1705" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Tessa.xp_to_next</x:v>
+      </x:c>
+      <x:c r="B1705" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1705" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1705" s="100" t="str">
+        <x:v>xp_events.001.results.Tessa.xp_to_next</x:v>
+      </x:c>
+      <x:c r="E1705" s="100" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="F1705" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1706" ht="30" customHeight="1">
+      <x:c r="A1706" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Owen.level</x:v>
+      </x:c>
+      <x:c r="B1706" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1706" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1706" s="96" t="str">
+        <x:v>xp_events.001.results.Owen.level</x:v>
+      </x:c>
+      <x:c r="E1706" s="96" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F1706" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1707" ht="32" customHeight="1">
+      <x:c r="A1707" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Owen.mana_current</x:v>
+      </x:c>
+      <x:c r="B1707" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1707" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1707" s="100" t="str">
+        <x:v>xp_events.001.results.Owen.mana_current</x:v>
+      </x:c>
+      <x:c r="E1707" s="100" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F1707" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1708" ht="30" customHeight="1">
+      <x:c r="A1708" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Owen.mana_max</x:v>
+      </x:c>
+      <x:c r="B1708" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1708" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1708" s="96" t="str">
+        <x:v>xp_events.001.results.Owen.mana_max</x:v>
+      </x:c>
+      <x:c r="E1708" s="96" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F1708" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1709" ht="30" customHeight="1">
+      <x:c r="A1709" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Owen.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="B1709" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1709" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1709" s="100" t="str">
+        <x:v>xp_events.001.results.Owen.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="E1709" s="100" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F1709" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1710" ht="30" customHeight="1">
+      <x:c r="A1710" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Owen.xp_to_next</x:v>
+      </x:c>
+      <x:c r="B1710" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1710" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1710" s="96" t="str">
+        <x:v>xp_events.001.results.Owen.xp_to_next</x:v>
+      </x:c>
+      <x:c r="E1710" s="96" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="F1710" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1711" ht="30" customHeight="1">
+      <x:c r="A1711" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Dane.level</x:v>
+      </x:c>
+      <x:c r="B1711" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1711" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1711" s="100" t="str">
+        <x:v>xp_events.001.results.Dane.level</x:v>
+      </x:c>
+      <x:c r="E1711" s="100" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F1711" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1712" ht="32" customHeight="1">
+      <x:c r="A1712" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Dane.mana_current</x:v>
+      </x:c>
+      <x:c r="B1712" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1712" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1712" s="96" t="str">
+        <x:v>xp_events.001.results.Dane.mana_current</x:v>
+      </x:c>
+      <x:c r="E1712" s="96" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F1712" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1713" ht="30" customHeight="1">
+      <x:c r="A1713" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Dane.mana_max</x:v>
+      </x:c>
+      <x:c r="B1713" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1713" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1713" s="100" t="str">
+        <x:v>xp_events.001.results.Dane.mana_max</x:v>
+      </x:c>
+      <x:c r="E1713" s="100" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F1713" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1714" ht="30" customHeight="1">
+      <x:c r="A1714" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.results.Dane.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="B1714" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1714" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1714" s="96" t="str">
+        <x:v>xp_events.001.results.Dane.xp_in_bar</x:v>
+      </x:c>
+      <x:c r="E1714" s="96" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F1714" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1715" ht="30" customHeight="1">
+      <x:c r="A1715" s="99" t="str">
+        <x:v>ACT-002-xp_events.001.results.Dane.xp_to_next</x:v>
+      </x:c>
+      <x:c r="B1715" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1715" s="99" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1715" s="100" t="str">
+        <x:v>xp_events.001.results.Dane.xp_to_next</x:v>
+      </x:c>
+      <x:c r="E1715" s="100" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="F1715" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1716" ht="30" customHeight="1">
+      <x:c r="A1716" s="95" t="str">
+        <x:v>ACT-002-xp_events.001.limits</x:v>
+      </x:c>
+      <x:c r="B1716" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1716" s="95" t="str">
+        <x:v>Actual xp_events</x:v>
+      </x:c>
+      <x:c r="D1716" s="96" t="str">
+        <x:v>xp_events.001.limits</x:v>
+      </x:c>
+      <x:c r="E1716" s="96" t="str">
+        <x:v>One award per person for this resolved retreat; no Jory award or hunter kill award established.</x:v>
+      </x:c>
+      <x:c r="F1716" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1717" ht="30" customHeight="1">
+      <x:c r="A1717" s="99" t="str">
+        <x:v>ACT-002-practice</x:v>
+      </x:c>
+      <x:c r="B1717" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1717" s="99" t="str">
+        <x:v>Actual practice</x:v>
+      </x:c>
+      <x:c r="D1717" s="100" t="str">
+        <x:v>practice</x:v>
+      </x:c>
+      <x:c r="E1717" s="100" t="str">
+        <x:v>No focused practice, rank change or class milestone completed.</x:v>
+      </x:c>
+      <x:c r="F1717" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1718" ht="32" customHeight="1">
+      <x:c r="A1718" s="95" t="str">
+        <x:v>ACT-002-injuries.001</x:v>
+      </x:c>
+      <x:c r="B1718" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1718" s="95" t="str">
+        <x:v>Actual injuries</x:v>
+      </x:c>
+      <x:c r="D1718" s="96" t="str">
+        <x:v>injuries.001</x:v>
+      </x:c>
+      <x:c r="E1718" s="96" t="str">
+        <x:v>Kip: superficial forearm cut closed by one complete Mend; residual tenderness and shoulder soreness remain. No blood replacement or general healing.</x:v>
+      </x:c>
+      <x:c r="F1718" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1719" ht="30" customHeight="1">
+      <x:c r="A1719" s="99" t="str">
+        <x:v>ACT-002-injuries.002</x:v>
+      </x:c>
+      <x:c r="B1719" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1719" s="99" t="str">
+        <x:v>Actual injuries</x:v>
+      </x:c>
+      <x:c r="D1719" s="100" t="str">
+        <x:v>injuries.002</x:v>
+      </x:c>
+      <x:c r="E1719" s="100" t="str">
+        <x:v>Jory: splinted lower-leg fracture persists; previously closed shin cut remains closed.</x:v>
+      </x:c>
+      <x:c r="F1719" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1720" ht="32" customHeight="1">
+      <x:c r="A1720" s="95" t="str">
+        <x:v>ACT-002-injuries.003</x:v>
+      </x:c>
+      <x:c r="B1720" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1720" s="95" t="str">
+        <x:v>Actual injuries</x:v>
+      </x:c>
+      <x:c r="D1720" s="96" t="str">
+        <x:v>injuries.003</x:v>
+      </x:c>
+      <x:c r="E1720" s="96" t="str">
+        <x:v>Hunter: still wounded by the spent bolt, alive when driven back; scraping withdraws outside the barred door. No kill established.</x:v>
+      </x:c>
+      <x:c r="F1720" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1721" ht="30" customHeight="1">
+      <x:c r="A1721" s="99" t="str">
+        <x:v>ACT-002-objects.001</x:v>
+      </x:c>
+      <x:c r="B1721" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1721" s="99" t="str">
+        <x:v>Actual objects</x:v>
+      </x:c>
+      <x:c r="D1721" s="100" t="str">
+        <x:v>objects.001</x:v>
+      </x:c>
+      <x:c r="E1721" s="100" t="str">
+        <x:v>Jory rests on his litter inside the chamber; splint retained and repositioned carefully.</x:v>
+      </x:c>
+      <x:c r="F1721" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1722" ht="32" customHeight="1">
+      <x:c r="A1722" s="95" t="str">
+        <x:v>ACT-002-objects.002</x:v>
+      </x:c>
+      <x:c r="B1722" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1722" s="95" t="str">
+        <x:v>Actual objects</x:v>
+      </x:c>
+      <x:c r="D1722" s="96" t="str">
+        <x:v>objects.002</x:v>
+      </x:c>
+      <x:c r="E1722" s="96" t="str">
+        <x:v>Tessa retrieves/retains her short spear after using both hands at the door; Dane retains sword in right hand. No new weapon for Kip.</x:v>
+      </x:c>
+      <x:c r="F1722" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1723" ht="30" customHeight="1">
+      <x:c r="A1723" s="99" t="str">
+        <x:v>ACT-002-objects.003</x:v>
+      </x:c>
+      <x:c r="B1723" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1723" s="99" t="str">
+        <x:v>Actual objects</x:v>
+      </x:c>
+      <x:c r="D1723" s="100" t="str">
+        <x:v>objects.003</x:v>
+      </x:c>
+      <x:c r="E1723" s="100" t="str">
+        <x:v>The first launcher remains empty; its single spent bolt was not recovered.</x:v>
+      </x:c>
+      <x:c r="F1723" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1724" ht="32" customHeight="1">
+      <x:c r="A1724" s="95" t="str">
+        <x:v>ACT-002-objects.004</x:v>
+      </x:c>
+      <x:c r="B1724" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1724" s="95" t="str">
+        <x:v>Actual objects</x:v>
+      </x:c>
+      <x:c r="D1724" s="96" t="str">
+        <x:v>objects.004</x:v>
+      </x:c>
+      <x:c r="E1724" s="96" t="str">
+        <x:v>Fire vent used through one full five-second Override; control ended normally. No ownership or permanent suppression established.</x:v>
+      </x:c>
+      <x:c r="F1724" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1725" ht="30" customHeight="1">
+      <x:c r="A1725" s="99" t="str">
+        <x:v>ACT-002-objects.005</x:v>
+      </x:c>
+      <x:c r="B1725" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1725" s="99" t="str">
+        <x:v>Actual objects</x:v>
+      </x:c>
+      <x:c r="D1725" s="100" t="str">
+        <x:v>objects.005</x:v>
+      </x:c>
+      <x:c r="E1725" s="100" t="str">
+        <x:v>Kip retains keys and wallet. His phone remains charging in the van on Earth.</x:v>
+      </x:c>
+      <x:c r="F1725" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1726" ht="32" customHeight="1">
+      <x:c r="A1726" s="95" t="str">
+        <x:v>ACT-002-knowledge.Kip.001</x:v>
+      </x:c>
+      <x:c r="B1726" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1726" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1726" s="96" t="str">
+        <x:v>knowledge.Kip.001</x:v>
+      </x:c>
+      <x:c r="E1726" s="96" t="str">
+        <x:v>Knows Dane Mercer is expedition leader and has a class; observed eight-second Bulwark reduce but not eliminate impacts.</x:v>
+      </x:c>
+      <x:c r="F1726" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1727" ht="32" customHeight="1">
+      <x:c r="A1727" s="99" t="str">
+        <x:v>ACT-002-knowledge.Kip.002</x:v>
+      </x:c>
+      <x:c r="B1727" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1727" s="99" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1727" s="100" t="str">
+        <x:v>knowledge.Kip.002</x:v>
+      </x:c>
+      <x:c r="E1727" s="100" t="str">
+        <x:v>Has demonstrated a second legal Override on a seven-metre visible fire vent with an ordinary pivot and safe firing arc.</x:v>
+      </x:c>
+      <x:c r="F1727" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1728" ht="32" customHeight="1">
+      <x:c r="A1728" s="95" t="str">
+        <x:v>ACT-002-knowledge.Kip.003</x:v>
+      </x:c>
+      <x:c r="B1728" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1728" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1728" s="96" t="str">
+        <x:v>knowledge.Kip.003</x:v>
+      </x:c>
+      <x:c r="E1728" s="96" t="str">
+        <x:v>Knows Mend takes twenty seconds and twenty Mana and cannot set Jory's broken bone. No full companion descriptions/private values learned.</x:v>
+      </x:c>
+      <x:c r="F1728" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1729" ht="32" customHeight="1">
+      <x:c r="A1729" s="99" t="str">
+        <x:v>ACT-002-knowledge.Kip.004</x:v>
+      </x:c>
+      <x:c r="B1729" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1729" s="99" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1729" s="100" t="str">
+        <x:v>knowledge.Kip.004</x:v>
+      </x:c>
+      <x:c r="E1729" s="100" t="str">
+        <x:v>Knows his own level two, XP zero of two hundred, Mana twenty of forty-five; leveling increased maximum without refilling current Mana or removing fatigue.</x:v>
+      </x:c>
+      <x:c r="F1729" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1730" ht="32" customHeight="1">
+      <x:c r="A1730" s="95" t="str">
+        <x:v>ACT-002-knowledge.Kip.005</x:v>
+      </x:c>
+      <x:c r="B1730" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1730" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1730" s="96" t="str">
+        <x:v>knowledge.Kip.005</x:v>
+      </x:c>
+      <x:c r="E1730" s="96" t="str">
+        <x:v>Knows Tessa, Owen and Dane received the same one-hundred XP reward after their linked retreat/rescue completed. No reward for Jory established.</x:v>
+      </x:c>
+      <x:c r="F1730" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1731" ht="32" customHeight="1">
+      <x:c r="A1731" s="99" t="str">
+        <x:v>ACT-002-knowledge.Kip.006</x:v>
+      </x:c>
+      <x:c r="B1731" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1731" s="99" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1731" s="100" t="str">
+        <x:v>knowledge.Kip.006</x:v>
+      </x:c>
+      <x:c r="E1731" s="100" t="str">
+        <x:v>Knows the room has a floor anchor; Claim Room remains unread/unselected. Does not yet know its cost, obligations or result.</x:v>
+      </x:c>
+      <x:c r="F1731" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1732" ht="32" customHeight="1">
+      <x:c r="A1732" s="95" t="str">
+        <x:v>ACT-002-knowledge.Tessa/Owen/Dane.001</x:v>
+      </x:c>
+      <x:c r="B1732" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1732" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1732" s="96" t="str">
+        <x:v>knowledge.Tessa/Owen/Dane.001</x:v>
+      </x:c>
+      <x:c r="E1732" s="96" t="str">
+        <x:v>Kip openly confirms he has a class and can turn/fire the vent for five seconds. He does not disclose class name, legendary rarity or private Mana maximum.</x:v>
+      </x:c>
+      <x:c r="F1732" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1733" ht="30" customHeight="1">
+      <x:c r="A1733" s="99" t="str">
+        <x:v>ACT-002-knowledge.Tessa/Owen/Dane.002</x:v>
+      </x:c>
+      <x:c r="B1733" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1733" s="99" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1733" s="100" t="str">
+        <x:v>knowledge.Tessa/Owen/Dane.002</x:v>
+      </x:c>
+      <x:c r="E1733" s="100" t="str">
+        <x:v>Kip has not yet introduced his own name or Earth biography aloud.</x:v>
+      </x:c>
+      <x:c r="F1733" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1734" ht="32" customHeight="1">
+      <x:c r="A1734" s="95" t="str">
+        <x:v>ACT-002-knowledge.Tessa/Owen/Dane.003</x:v>
+      </x:c>
+      <x:c r="B1734" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1734" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1734" s="96" t="str">
+        <x:v>knowledge.Tessa/Owen/Dane.003</x:v>
+      </x:c>
+      <x:c r="E1734" s="96" t="str">
+        <x:v>The four active contributors confirm the same retreat award; their different levels need not rise together.</x:v>
+      </x:c>
+      <x:c r="F1734" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1735" ht="32" customHeight="1">
+      <x:c r="A1735" s="99" t="str">
+        <x:v>ACT-002-knowledge.reader.001</x:v>
+      </x:c>
+      <x:c r="B1735" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1735" s="99" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1735" s="100" t="str">
+        <x:v>knowledge.reader.001</x:v>
+      </x:c>
+      <x:c r="E1735" s="100" t="str">
+        <x:v>Noah is Kip's nineteen-year-old younger brother with his own life at home; this is Kip's private worry, not information shared with companions.</x:v>
+      </x:c>
+      <x:c r="F1735" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1736" ht="32" customHeight="1">
+      <x:c r="A1736" s="95" t="str">
+        <x:v>ACT-002-knowledge.reader.002</x:v>
+      </x:c>
+      <x:c r="B1736" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1736" s="95" t="str">
+        <x:v>Actual knowledge</x:v>
+      </x:c>
+      <x:c r="D1736" s="96" t="str">
+        <x:v>knowledge.reader.002</x:v>
+      </x:c>
+      <x:c r="E1736" s="96" t="str">
+        <x:v>The hunter withdrew audibly, not a confirmed kill; the room is temporary physical shelter with an untested anchor.</x:v>
+      </x:c>
+      <x:c r="F1736" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1737" ht="32" customHeight="1">
+      <x:c r="A1737" s="99" t="str">
+        <x:v>ACT-002-private_flags.001</x:v>
+      </x:c>
+      <x:c r="B1737" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1737" s="99" t="str">
+        <x:v>Actual private_flags</x:v>
+      </x:c>
+      <x:c r="D1737" s="100" t="str">
+        <x:v>private_flags.001</x:v>
+      </x:c>
+      <x:c r="E1737" s="100" t="str">
+        <x:v>Current companion levels, reserves and ability versions carry approved author baselines reconciled with actual paid uses; they are not all disclosed in dialogue.</x:v>
+      </x:c>
+      <x:c r="F1737" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1738" ht="32" customHeight="1">
+      <x:c r="A1738" s="95" t="str">
+        <x:v>ACT-002-private_flags.002</x:v>
+      </x:c>
+      <x:c r="B1738" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1738" s="95" t="str">
+        <x:v>Actual private_flags</x:v>
+      </x:c>
+      <x:c r="D1738" s="96" t="str">
+        <x:v>private_flags.002</x:v>
+      </x:c>
+      <x:c r="E1738" s="96" t="str">
+        <x:v>Each of the four material contributors receives the retreat challenge award once. No kill award or second reward for patient repositioning.</x:v>
+      </x:c>
+      <x:c r="F1738" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1739" ht="32" customHeight="1">
+      <x:c r="A1739" s="99" t="str">
+        <x:v>ACT-002-private_flags.003</x:v>
+      </x:c>
+      <x:c r="B1739" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1739" s="99" t="str">
+        <x:v>Actual private_flags</x:v>
+      </x:c>
+      <x:c r="D1739" s="100" t="str">
+        <x:v>private_flags.003</x:v>
+      </x:c>
+      <x:c r="E1739" s="100" t="str">
+        <x:v>Several minutes of active care/checks do not establish sitting/lying uninterrupted recovery; no rest credit is applied.</x:v>
+      </x:c>
+      <x:c r="F1739" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1740" ht="30" customHeight="1">
+      <x:c r="A1740" s="95" t="str">
+        <x:v>ACT-002-private_flags.004</x:v>
+      </x:c>
+      <x:c r="B1740" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1740" s="95" t="str">
+        <x:v>Actual private_flags</x:v>
+      </x:c>
+      <x:c r="D1740" s="96" t="str">
+        <x:v>private_flags.004</x:v>
+      </x:c>
+      <x:c r="E1740" s="96" t="str">
+        <x:v>Kip's name remains to be introduced aloud before others can address him by it.</x:v>
+      </x:c>
+      <x:c r="F1740" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1741" ht="32" customHeight="1">
+      <x:c r="A1741" s="99" t="str">
+        <x:v>ACT-002-private_flags.005</x:v>
+      </x:c>
+      <x:c r="B1741" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1741" s="99" t="str">
+        <x:v>Actual private_flags</x:v>
+      </x:c>
+      <x:c r="D1741" s="100" t="str">
+        <x:v>private_flags.005</x:v>
+      </x:c>
+      <x:c r="E1741" s="100" t="str">
+        <x:v>Actual floor anchor and fallen-stone service blockage govern the next episode, overriding older planned inner-wall/bar wording.</x:v>
+      </x:c>
+      <x:c r="F1741" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1742" ht="48" customHeight="1">
+      <x:c r="A1742" s="95" t="str">
+        <x:v>ACT-002-ending</x:v>
+      </x:c>
+      <x:c r="B1742" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1742" s="95" t="str">
+        <x:v>Actual ending</x:v>
+      </x:c>
+      <x:c r="D1742" s="96" t="str">
+        <x:v>ending</x:v>
+      </x:c>
+      <x:c r="E1742" s="96" t="str">
+        <x:v>All five are physically sheltered in the barred service chamber, with the onward passage obstructed. Kip has twenty Mana and considers inspecting Claim Room before committing; no room claimed or new skill granted.</x:v>
+      </x:c>
+      <x:c r="F1742" s="96" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1743" ht="30" customHeight="1">
+      <x:c r="A1743" s="99" t="str">
+        <x:v>ACT-002-open_issues</x:v>
+      </x:c>
+      <x:c r="B1743" s="99" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C1743" s="99" t="str">
+        <x:v>Actual open_issues</x:v>
+      </x:c>
+      <x:c r="D1743" s="100" t="str">
+        <x:v>open_issues</x:v>
+      </x:c>
+      <x:c r="E1743" s="100" t="str">
+        <x:v>None recorded</x:v>
+      </x:c>
+      <x:c r="F1743" s="100" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F8:F1459">
     <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Open"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ecf394ac354926"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39055cfe1dbb44d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52219,7 +55553,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>Confirmed through Episode 1: Legendary, Level One.</x:v>
+        <x:v>Confirmed through Episode 2: Twenty Mana Left.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -52257,7 +55591,7 @@
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="88" t="str">
-        <x:v>Stopping point: All five remain alive and in retreat beyond the junction. Kip and Owen carry Jory toward the service-door bend while the rearguard delays the living wounded hunter; no refuge or escape is secured.</x:v>
+        <x:v>Stopping point: All five are physically sheltered in the barred service chamber, with the onward passage obstructed. Kip has twenty Mana and considers inspecting Claim Room before committing; no room claimed or new skill granted.</x:v>
       </x:c>
       <x:c r="B6" s="88"/>
       <x:c r="C6" s="88"/>
@@ -52491,69 +55825,179 @@
         <x:v>2026-10-22T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="70"/>
-      <x:c r="B12" s="64"/>
-      <x:c r="C12" s="70"/>
-      <x:c r="D12" s="70"/>
-      <x:c r="E12" s="70"/>
-      <x:c r="F12" s="70"/>
-      <x:c r="G12" s="70"/>
-      <x:c r="H12" s="64"/>
-      <x:c r="I12" s="65"/>
-      <x:c r="J12" s="65"/>
-      <x:c r="K12" s="65"/>
-      <x:c r="L12" s="65"/>
-      <x:c r="M12" s="64"/>
-      <x:c r="N12" s="72"/>
-    </x:row>
-    <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="70"/>
-      <x:c r="B13" s="64"/>
-      <x:c r="C13" s="70"/>
-      <x:c r="D13" s="70"/>
-      <x:c r="E13" s="70"/>
-      <x:c r="F13" s="70"/>
-      <x:c r="G13" s="70"/>
-      <x:c r="H13" s="64"/>
-      <x:c r="I13" s="65"/>
-      <x:c r="J13" s="65"/>
-      <x:c r="K13" s="65"/>
-      <x:c r="L13" s="65"/>
-      <x:c r="M13" s="64"/>
-      <x:c r="N13" s="72"/>
-    </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="70"/>
-      <x:c r="B14" s="64"/>
-      <x:c r="C14" s="70"/>
-      <x:c r="D14" s="70"/>
-      <x:c r="E14" s="70"/>
-      <x:c r="F14" s="70"/>
-      <x:c r="G14" s="70"/>
-      <x:c r="H14" s="64"/>
-      <x:c r="I14" s="65"/>
-      <x:c r="J14" s="65"/>
-      <x:c r="K14" s="65"/>
-      <x:c r="L14" s="65"/>
-      <x:c r="M14" s="64"/>
-      <x:c r="N14" s="72"/>
-    </x:row>
-    <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="70"/>
-      <x:c r="B15" s="64"/>
-      <x:c r="C15" s="70"/>
-      <x:c r="D15" s="70"/>
-      <x:c r="E15" s="70"/>
-      <x:c r="F15" s="70"/>
-      <x:c r="G15" s="70"/>
-      <x:c r="H15" s="64"/>
-      <x:c r="I15" s="65"/>
-      <x:c r="J15" s="65"/>
-      <x:c r="K15" s="65"/>
-      <x:c r="L15" s="65"/>
-      <x:c r="M15" s="64"/>
-      <x:c r="N15" s="72"/>
+    <x:row r="12" ht="70" customHeight="1">
+      <x:c r="A12" s="89" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B12" s="90" t="str">
+        <x:v>Kip</x:v>
+      </x:c>
+      <x:c r="C12" s="89" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D12" s="89" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E12" s="89" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F12" s="89" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="89" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="H12" s="90" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I12" s="91" t="str">
+        <x:v>Kip: superficial forearm cut closed by one complete Mend; residual tenderness and shoulder soreness remain. No blood replacement or general healing.</x:v>
+      </x:c>
+      <x:c r="J12" s="91" t="str">
+        <x:v>See actual Episode 2 knowledge facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="K12" s="91" t="str">
+        <x:v>See actual Episode 2 custody facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="L12" s="91" t="str">
+        <x:v>chapters/chapter-01/episode-002.txt
+SHA-256 be408ba46776ec799bef78564c6ba621f3193fc6bf9c10d2a66dd2e29f18202b</x:v>
+      </x:c>
+      <x:c r="M12" s="90" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+      <x:c r="N12" s="92" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="70" customHeight="1">
+      <x:c r="A13" s="89" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B13" s="90" t="str">
+        <x:v>Tessa</x:v>
+      </x:c>
+      <x:c r="C13" s="89" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D13" s="89" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E13" s="89" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F13" s="89" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G13" s="89" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="H13" s="90" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I13" s="91"/>
+      <x:c r="J13" s="91" t="str">
+        <x:v>See actual Episode 2 knowledge facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="K13" s="91" t="str">
+        <x:v>See actual Episode 2 custody facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="L13" s="91" t="str">
+        <x:v>chapters/chapter-01/episode-002.txt
+SHA-256 be408ba46776ec799bef78564c6ba621f3193fc6bf9c10d2a66dd2e29f18202b</x:v>
+      </x:c>
+      <x:c r="M13" s="90" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+      <x:c r="N13" s="92" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="70" customHeight="1">
+      <x:c r="A14" s="89" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B14" s="90" t="str">
+        <x:v>Owen</x:v>
+      </x:c>
+      <x:c r="C14" s="89" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D14" s="89" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E14" s="89" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F14" s="89" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G14" s="89" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="H14" s="90" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I14" s="91"/>
+      <x:c r="J14" s="91" t="str">
+        <x:v>See actual Episode 2 knowledge facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="K14" s="91" t="str">
+        <x:v>See actual Episode 2 custody facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="L14" s="91" t="str">
+        <x:v>chapters/chapter-01/episode-002.txt
+SHA-256 be408ba46776ec799bef78564c6ba621f3193fc6bf9c10d2a66dd2e29f18202b</x:v>
+      </x:c>
+      <x:c r="M14" s="90" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+      <x:c r="N14" s="92" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="89" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B15" s="90" t="str">
+        <x:v>Dane</x:v>
+      </x:c>
+      <x:c r="C15" s="89" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D15" s="89" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E15" s="89" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F15" s="89" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G15" s="89" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="H15" s="90" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I15" s="91"/>
+      <x:c r="J15" s="91" t="str">
+        <x:v>See actual Episode 2 knowledge facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="K15" s="91" t="str">
+        <x:v>See actual Episode 2 custody facts in Story carryover.</x:v>
+      </x:c>
+      <x:c r="L15" s="91" t="str">
+        <x:v>chapters/chapter-01/episode-002.txt
+SHA-256 be408ba46776ec799bef78564c6ba621f3193fc6bf9c10d2a66dd2e29f18202b</x:v>
+      </x:c>
+      <x:c r="M15" s="90" t="str">
+        <x:v>Confirmed from final text</x:v>
+      </x:c>
+      <x:c r="N15" s="92" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="70"/>
@@ -52903,9 +56347,12 @@
     <x:cfRule type="expression" dxfId="6" priority="2">
       <x:formula>AND($M8="Confirmed from final text",$L8="")</x:formula>
     </x:cfRule>
+    <x:cfRule type="expression" dxfId="7" priority="3">
+      <x:formula>AND($M8="Confirmed from final text",$L8="")</x:formula>
+    </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="5">
-    <x:dataValidation type="list" sqref="M12:M27">
+  <x:dataValidations count="9">
+    <x:dataValidation type="list" sqref="M16:M27">
       <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="M8">
@@ -52920,10 +56367,22 @@
     <x:dataValidation type="list" sqref="M11">
       <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="M12">
+      <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M13">
+      <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M14">
+      <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M15">
+      <x:formula1>"Needs final-text review,Confirmed from final text,Superseded"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reacb95c8c24a43df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra45895ef6b98486a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53846,7 +57305,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc5e9584ed554c91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e07407494b9492f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>